<commit_message>
Ulepsz filtrowanie nowości i podgląd kart
</commit_message>
<xml_diff>
--- a/KONSPEKT - FINGERSTYLE.xlsx
+++ b/KONSPEKT - FINGERSTYLE.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BAZA" sheetId="1" r:id="Rd6fde7a4742c46b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BAZA" sheetId="1" r:id="R11ac84c3202a4add"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -653,8 +653,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
+    <x:numFmt numFmtId="200" formatCode="@"/>
   </x:numFmts>
   <x:fonts count="3">
     <x:font>
@@ -686,7 +687,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="12">
+  <x:cellXfs count="13">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
@@ -715,6 +716,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="2">
     <x:cellStyle name="Normal" xfId="1"/>
@@ -724,19 +726,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Baza_FINGERSTYLE" displayName="Baza_FINGERSTYLE" ref="A1:J70" totalsRowShown="0">
-  <x:autoFilter ref="A1:J70"/>
-  <x:tableColumns count="10">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Baza_FINGERSTYLE" displayName="Baza_FINGERSTYLE" ref="A1:K70" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:K70"/>
+  <x:tableColumns count="11">
     <x:tableColumn id="1" name="UTWÓR"/>
     <x:tableColumn id="2" name="WYKONAWCA"/>
     <x:tableColumn id="3" name="POZIOM"/>
-    <x:tableColumn id="5" name="OPIS"/>
-    <x:tableColumn id="6" name="TAGI"/>
-    <x:tableColumn id="7" name="RODZAJ OPRACOWANIA"/>
-    <x:tableColumn id="8" name="KATEGORIE DODATKOWE"/>
-    <x:tableColumn id="9" name="YOUTUBE"/>
-    <x:tableColumn id="10" name="LINK DO DYSKU"/>
-    <x:tableColumn id="11" name="DATA"/>
+    <x:tableColumn id="4" name="OPIS"/>
+    <x:tableColumn id="5" name="TAGI"/>
+    <x:tableColumn id="6" name="RODZAJ OPRACOWANIA"/>
+    <x:tableColumn id="7" name="KATEGORIE DODATKOWE"/>
+    <x:tableColumn id="8" name="YOUTUBE"/>
+    <x:tableColumn id="9" name="LINK DO DYSKU"/>
+    <x:tableColumn id="10" name="DATA"/>
+    <x:tableColumn id="11" name="ID"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -945,6 +948,7 @@
     <x:col min="8" max="8" width="12" customWidth="1"/>
     <x:col min="9" max="9" width="64" customWidth="1"/>
     <x:col min="10" max="10" width="14" customWidth="1"/>
+    <x:col min="11" max="11" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -978,6 +982,9 @@
       <x:c r="J1" t="s">
         <x:v>9</x:v>
       </x:c>
+      <x:c r="K1" s="12" t="str">
+        <x:v>ID</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="1" t="s">
@@ -999,6 +1006,9 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="J2" s="2"/>
+      <x:c r="K2" s="12" t="str">
+        <x:v>UTW-0055</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1" t="s">
@@ -1023,6 +1033,9 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="J3" s="2"/>
+      <x:c r="K3" s="12" t="str">
+        <x:v>UTW-0056</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="1" t="s">
@@ -1044,6 +1057,9 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="J4" s="2"/>
+      <x:c r="K4" s="12" t="str">
+        <x:v>UTW-0057</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="1" t="s">
@@ -1068,6 +1084,9 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="J5" s="2"/>
+      <x:c r="K5" s="12" t="str">
+        <x:v>UTW-0058</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="1" t="s">
@@ -1092,6 +1111,9 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="J6" s="2"/>
+      <x:c r="K6" s="12" t="str">
+        <x:v>UTW-0059</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="1" t="s">
@@ -1113,6 +1135,9 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="J7" s="2"/>
+      <x:c r="K7" s="12" t="str">
+        <x:v>UTW-0060</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="1" t="s">
@@ -1134,6 +1159,9 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="J8" s="2"/>
+      <x:c r="K8" s="12" t="str">
+        <x:v>UTW-0061</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="1" t="s">
@@ -1158,6 +1186,9 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="J9" s="2"/>
+      <x:c r="K9" s="12" t="str">
+        <x:v>UTW-0062</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="1" t="s">
@@ -1179,6 +1210,9 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="J10" s="2"/>
+      <x:c r="K10" s="12" t="str">
+        <x:v>UTW-0063</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="1" t="s">
@@ -1200,6 +1234,9 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="J11" s="2"/>
+      <x:c r="K11" s="12" t="str">
+        <x:v>UTW-0064</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="1" t="s">
@@ -1221,6 +1258,9 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="J12" s="2"/>
+      <x:c r="K12" s="12" t="str">
+        <x:v>UTW-0065</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="1" t="s">
@@ -1245,6 +1285,9 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="J13" s="2"/>
+      <x:c r="K13" s="12" t="str">
+        <x:v>UTW-0066</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="1" t="s">
@@ -1266,6 +1309,9 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="J14" s="2"/>
+      <x:c r="K14" s="12" t="str">
+        <x:v>UTW-0067</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="1" t="s">
@@ -1287,6 +1333,9 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="J15" s="2"/>
+      <x:c r="K15" s="12" t="str">
+        <x:v>UTW-0068</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="1" t="s">
@@ -1311,6 +1360,9 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="J16" s="2"/>
+      <x:c r="K16" s="12" t="str">
+        <x:v>UTW-0069</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="1" t="s">
@@ -1332,6 +1384,9 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="J17" s="2"/>
+      <x:c r="K17" s="12" t="str">
+        <x:v>UTW-0070</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="1" t="s">
@@ -1353,6 +1408,9 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="J18" s="2"/>
+      <x:c r="K18" s="12" t="str">
+        <x:v>UTW-0071</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="1" t="s">
@@ -1374,6 +1432,9 @@
         <x:v>68</x:v>
       </x:c>
       <x:c r="J19" s="2"/>
+      <x:c r="K19" s="12" t="str">
+        <x:v>UTW-0072</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="1" t="s">
@@ -1395,6 +1456,9 @@
         <x:v>72</x:v>
       </x:c>
       <x:c r="J20" s="2"/>
+      <x:c r="K20" s="12" t="str">
+        <x:v>UTW-0073</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="1" t="s">
@@ -1419,6 +1483,9 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="J21" s="2"/>
+      <x:c r="K21" s="12" t="str">
+        <x:v>UTW-0074</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="1" t="s">
@@ -1440,6 +1507,9 @@
         <x:v>78</x:v>
       </x:c>
       <x:c r="J22" s="2"/>
+      <x:c r="K22" s="12" t="str">
+        <x:v>UTW-0075</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="1" t="s">
@@ -1461,6 +1531,9 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="J23" s="2"/>
+      <x:c r="K23" s="12" t="str">
+        <x:v>UTW-0076</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="1" t="s">
@@ -1485,6 +1558,9 @@
         <x:v>83</x:v>
       </x:c>
       <x:c r="J24" s="2"/>
+      <x:c r="K24" s="12" t="str">
+        <x:v>UTW-0077</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="1" t="s">
@@ -1506,6 +1582,9 @@
         <x:v>85</x:v>
       </x:c>
       <x:c r="J25" s="2"/>
+      <x:c r="K25" s="12" t="str">
+        <x:v>UTW-0078</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="1" t="s">
@@ -1527,6 +1606,9 @@
         <x:v>88</x:v>
       </x:c>
       <x:c r="J26" s="2"/>
+      <x:c r="K26" s="12" t="str">
+        <x:v>UTW-0079</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="1" t="s">
@@ -1548,6 +1630,9 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="J27" s="2"/>
+      <x:c r="K27" s="12" t="str">
+        <x:v>UTW-0080</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="1" t="s">
@@ -1572,6 +1657,9 @@
         <x:v>93</x:v>
       </x:c>
       <x:c r="J28" s="2"/>
+      <x:c r="K28" s="12" t="str">
+        <x:v>UTW-0081</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="1" t="s">
@@ -1593,6 +1681,9 @@
         <x:v>96</x:v>
       </x:c>
       <x:c r="J29" s="2"/>
+      <x:c r="K29" s="12" t="str">
+        <x:v>UTW-0082</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="1" t="s">
@@ -1617,6 +1708,9 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="J30" s="2"/>
+      <x:c r="K30" s="12" t="str">
+        <x:v>UTW-0083</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="1" t="s">
@@ -1641,6 +1735,9 @@
         <x:v>101</x:v>
       </x:c>
       <x:c r="J31" s="2"/>
+      <x:c r="K31" s="12" t="str">
+        <x:v>UTW-0084</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="1" t="s">
@@ -1662,6 +1759,9 @@
         <x:v>104</x:v>
       </x:c>
       <x:c r="J32" s="2"/>
+      <x:c r="K32" s="12" t="str">
+        <x:v>UTW-0085</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="1" t="s">
@@ -1683,6 +1783,9 @@
         <x:v>107</x:v>
       </x:c>
       <x:c r="J33" s="2"/>
+      <x:c r="K33" s="12" t="str">
+        <x:v>UTW-0086</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="1" t="s">
@@ -1704,6 +1807,9 @@
         <x:v>110</x:v>
       </x:c>
       <x:c r="J34" s="2"/>
+      <x:c r="K34" s="12" t="str">
+        <x:v>UTW-0087</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="1" t="s">
@@ -1725,6 +1831,9 @@
         <x:v>113</x:v>
       </x:c>
       <x:c r="J35" s="2"/>
+      <x:c r="K35" s="12" t="str">
+        <x:v>UTW-0088</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="1" t="s">
@@ -1749,6 +1858,9 @@
         <x:v>116</x:v>
       </x:c>
       <x:c r="J36" s="2"/>
+      <x:c r="K36" s="12" t="str">
+        <x:v>UTW-0089</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="1" t="s">
@@ -1773,6 +1885,9 @@
         <x:v>119</x:v>
       </x:c>
       <x:c r="J37" s="2"/>
+      <x:c r="K37" s="12" t="str">
+        <x:v>UTW-0090</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="1" t="s">
@@ -1797,6 +1912,9 @@
         <x:v>122</x:v>
       </x:c>
       <x:c r="J38" s="2"/>
+      <x:c r="K38" s="12" t="str">
+        <x:v>UTW-0091</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="1" t="s">
@@ -1818,6 +1936,9 @@
         <x:v>125</x:v>
       </x:c>
       <x:c r="J39" s="2"/>
+      <x:c r="K39" s="12" t="str">
+        <x:v>UTW-0092</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="1" t="s">
@@ -1842,6 +1963,9 @@
         <x:v>128</x:v>
       </x:c>
       <x:c r="J40" s="2"/>
+      <x:c r="K40" s="12" t="str">
+        <x:v>UTW-0093</x:v>
+      </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="1" t="s">
@@ -1866,6 +1990,9 @@
         <x:v>131</x:v>
       </x:c>
       <x:c r="J41" s="2"/>
+      <x:c r="K41" s="12" t="str">
+        <x:v>UTW-0094</x:v>
+      </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="1" t="s">
@@ -1890,6 +2017,9 @@
         <x:v>134</x:v>
       </x:c>
       <x:c r="J42" s="2"/>
+      <x:c r="K42" s="12" t="str">
+        <x:v>UTW-0095</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="1" t="s">
@@ -1911,6 +2041,9 @@
         <x:v>136</x:v>
       </x:c>
       <x:c r="J43" s="2"/>
+      <x:c r="K43" s="12" t="str">
+        <x:v>UTW-0096</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="1" t="s">
@@ -1932,6 +2065,9 @@
         <x:v>139</x:v>
       </x:c>
       <x:c r="J44" s="2"/>
+      <x:c r="K44" s="12" t="str">
+        <x:v>UTW-0097</x:v>
+      </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="1" t="s">
@@ -1953,6 +2089,9 @@
         <x:v>142</x:v>
       </x:c>
       <x:c r="J45" s="2"/>
+      <x:c r="K45" s="12" t="str">
+        <x:v>UTW-0098</x:v>
+      </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="1" t="s">
@@ -1974,6 +2113,9 @@
         <x:v>145</x:v>
       </x:c>
       <x:c r="J46" s="2"/>
+      <x:c r="K46" s="12" t="str">
+        <x:v>UTW-0099</x:v>
+      </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="1" t="s">
@@ -1998,6 +2140,9 @@
         <x:v>148</x:v>
       </x:c>
       <x:c r="J47" s="2"/>
+      <x:c r="K47" s="12" t="str">
+        <x:v>UTW-0100</x:v>
+      </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="1" t="s">
@@ -2022,6 +2167,9 @@
         <x:v>150</x:v>
       </x:c>
       <x:c r="J48" s="2"/>
+      <x:c r="K48" s="12" t="str">
+        <x:v>UTW-0101</x:v>
+      </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="1" t="s">
@@ -2043,6 +2191,9 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="J49" s="2"/>
+      <x:c r="K49" s="12" t="str">
+        <x:v>UTW-0102</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="1" t="s">
@@ -2067,6 +2218,9 @@
         <x:v>155</x:v>
       </x:c>
       <x:c r="J50" s="2"/>
+      <x:c r="K50" s="12" t="str">
+        <x:v>UTW-0103</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="1" t="s">
@@ -2088,6 +2242,9 @@
         <x:v>158</x:v>
       </x:c>
       <x:c r="J51" s="2"/>
+      <x:c r="K51" s="12" t="str">
+        <x:v>UTW-0104</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="1" t="s">
@@ -2112,6 +2269,9 @@
         <x:v>161</x:v>
       </x:c>
       <x:c r="J52" s="2"/>
+      <x:c r="K52" s="12" t="str">
+        <x:v>UTW-0105</x:v>
+      </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="1" t="s">
@@ -2133,6 +2293,9 @@
         <x:v>164</x:v>
       </x:c>
       <x:c r="J53" s="2"/>
+      <x:c r="K53" s="12" t="str">
+        <x:v>UTW-0106</x:v>
+      </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="1" t="s">
@@ -2154,6 +2317,9 @@
         <x:v>167</x:v>
       </x:c>
       <x:c r="J54" s="2"/>
+      <x:c r="K54" s="12" t="str">
+        <x:v>UTW-0107</x:v>
+      </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="1" t="s">
@@ -2175,6 +2341,9 @@
         <x:v>169</x:v>
       </x:c>
       <x:c r="J55" s="2"/>
+      <x:c r="K55" s="12" t="str">
+        <x:v>UTW-0108</x:v>
+      </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="1" t="s">
@@ -2196,6 +2365,9 @@
         <x:v>172</x:v>
       </x:c>
       <x:c r="J56" s="2"/>
+      <x:c r="K56" s="12" t="str">
+        <x:v>UTW-0109</x:v>
+      </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="1" t="s">
@@ -2217,6 +2389,9 @@
         <x:v>175</x:v>
       </x:c>
       <x:c r="J57" s="2"/>
+      <x:c r="K57" s="12" t="str">
+        <x:v>UTW-0110</x:v>
+      </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="1" t="s">
@@ -2238,6 +2413,9 @@
         <x:v>178</x:v>
       </x:c>
       <x:c r="J58" s="2"/>
+      <x:c r="K58" s="12" t="str">
+        <x:v>UTW-0111</x:v>
+      </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="1" t="s">
@@ -2259,6 +2437,9 @@
         <x:v>181</x:v>
       </x:c>
       <x:c r="J59" s="2"/>
+      <x:c r="K59" s="12" t="str">
+        <x:v>UTW-0112</x:v>
+      </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="1" t="s">
@@ -2283,6 +2464,9 @@
         <x:v>184</x:v>
       </x:c>
       <x:c r="J60" s="2"/>
+      <x:c r="K60" s="12" t="str">
+        <x:v>UTW-0113</x:v>
+      </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="1" t="s">
@@ -2307,6 +2491,9 @@
         <x:v>186</x:v>
       </x:c>
       <x:c r="J61" s="2"/>
+      <x:c r="K61" s="12" t="str">
+        <x:v>UTW-0114</x:v>
+      </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="1" t="s">
@@ -2328,6 +2515,9 @@
         <x:v>189</x:v>
       </x:c>
       <x:c r="J62" s="2"/>
+      <x:c r="K62" s="12" t="str">
+        <x:v>UTW-0115</x:v>
+      </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="1" t="s">
@@ -2349,6 +2539,9 @@
         <x:v>192</x:v>
       </x:c>
       <x:c r="J63" s="2"/>
+      <x:c r="K63" s="12" t="str">
+        <x:v>UTW-0116</x:v>
+      </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="1" t="s">
@@ -2373,6 +2566,9 @@
         <x:v>195</x:v>
       </x:c>
       <x:c r="J64" s="2"/>
+      <x:c r="K64" s="12" t="str">
+        <x:v>UTW-0117</x:v>
+      </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="1" t="s">
@@ -2397,6 +2593,9 @@
         <x:v>197</x:v>
       </x:c>
       <x:c r="J65" s="2"/>
+      <x:c r="K65" s="12" t="str">
+        <x:v>UTW-0118</x:v>
+      </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="1" t="s">
@@ -2421,6 +2620,9 @@
         <x:v>200</x:v>
       </x:c>
       <x:c r="J66" s="2"/>
+      <x:c r="K66" s="12" t="str">
+        <x:v>UTW-0119</x:v>
+      </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="1" t="s">
@@ -2442,6 +2644,9 @@
         <x:v>203</x:v>
       </x:c>
       <x:c r="J67" s="2"/>
+      <x:c r="K67" s="12" t="str">
+        <x:v>UTW-0120</x:v>
+      </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="1" t="s">
@@ -2463,6 +2668,9 @@
         <x:v>206</x:v>
       </x:c>
       <x:c r="J68" s="2"/>
+      <x:c r="K68" s="12" t="str">
+        <x:v>UTW-0121</x:v>
+      </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="1" t="s">
@@ -2487,6 +2695,9 @@
         <x:v>209</x:v>
       </x:c>
       <x:c r="J69" s="2"/>
+      <x:c r="K69" s="12" t="str">
+        <x:v>UTW-0122</x:v>
+      </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="1" t="s">
@@ -2511,11 +2722,14 @@
         <x:v>212</x:v>
       </x:c>
       <x:c r="J70" s="2"/>
+      <x:c r="K70" s="12" t="str">
+        <x:v>UTW-0123</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54b64b05233b414e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refc17e00ccdd4001"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>